<commit_message>
Implement add new user with refactor the code
</commit_message>
<xml_diff>
--- a/src/main/resources/data/DB.xlsx
+++ b/src/main/resources/data/DB.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28730"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4a765bfb693053ce/Desktop/SecurePrints/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="635" documentId="13_ncr:1_{1D354D38-737B-4D3A-A9B1-62F2684C3BE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{15F6B4CD-678D-49FF-8DF1-C4AFA7A79AA9}"/>
+  <xr:revisionPtr revIDLastSave="646" documentId="13_ncr:1_{1D354D38-737B-4D3A-A9B1-62F2684C3BE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{64F969F8-109A-4EB0-803A-2A06D84C943A}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="810" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="810" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ServiceType" sheetId="5" r:id="rId1"/>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="200" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="203" uniqueCount="104">
   <si>
     <t>varchar(30)</t>
   </si>
@@ -112,9 +112,6 @@
     <t>BCI_FBI</t>
   </si>
   <si>
-    <t>rsn_text</t>
-  </si>
-  <si>
     <t>rsn_code</t>
   </si>
   <si>
@@ -226,12 +223,6 @@
     <t>Rent</t>
   </si>
   <si>
-    <t>bci_rsn_text</t>
-  </si>
-  <si>
-    <t>fbi_rsn_text</t>
-  </si>
-  <si>
     <t>appt_sts_code</t>
   </si>
   <si>
@@ -304,9 +295,6 @@
     <t>com_phone</t>
   </si>
   <si>
-    <t>comp_email</t>
-  </si>
-  <si>
     <t>com_id</t>
   </si>
   <si>
@@ -356,6 +344,21 @@
   </si>
   <si>
     <t>exp_pymt_sts_code</t>
+  </si>
+  <si>
+    <t>com_email</t>
+  </si>
+  <si>
+    <t>rsn_desc</t>
+  </si>
+  <si>
+    <t>bci_rsn_desc</t>
+  </si>
+  <si>
+    <t>fbi_rsn_desc</t>
+  </si>
+  <si>
+    <t>bci_amt</t>
   </si>
 </sst>
 </file>
@@ -706,14 +709,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B49DD3CD-B9FF-44D4-941A-E23CBF5677F3}">
-  <dimension ref="A2:C4"/>
+  <dimension ref="A2:D4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="2"/>
     <col min="2" max="2" width="28.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>18</v>
       </c>
@@ -723,8 +726,11 @@
       <c r="C2" s="1">
         <v>38</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D2" s="1">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>19</v>
       </c>
@@ -734,16 +740,22 @@
       <c r="C3" s="1">
         <v>48</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D3" s="1">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C4" s="1">
         <v>68</v>
+      </c>
+      <c r="D4" s="1">
+        <v>40</v>
       </c>
     </row>
   </sheetData>
@@ -753,7 +765,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{499D205C-AB14-4D61-B52D-6BDE054EBB20}">
-  <dimension ref="A2:C9"/>
+  <dimension ref="A2:C10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20.85546875" customWidth="1"/>
@@ -763,7 +775,7 @@
   <sheetData>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B2" t="s">
         <v>9</v>
@@ -774,7 +786,7 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B3" t="s">
         <v>9</v>
@@ -785,10 +797,10 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C4" t="s">
         <v>5</v>
@@ -796,10 +808,10 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="B5" t="s">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="C5" t="s">
         <v>5</v>
@@ -807,7 +819,7 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="B6" t="s">
         <v>8</v>
@@ -818,10 +830,10 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>47</v>
+        <v>91</v>
       </c>
       <c r="B7" t="s">
-        <v>43</v>
+        <v>8</v>
       </c>
       <c r="C7" t="s">
         <v>5</v>
@@ -829,24 +841,35 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>75</v>
+        <v>46</v>
       </c>
       <c r="B8" t="s">
-        <v>57</v>
+        <v>42</v>
       </c>
       <c r="C8" t="s">
-        <v>45</v>
+        <v>5</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="B9" t="s">
-        <v>43</v>
+        <v>56</v>
       </c>
       <c r="C9" t="s">
-        <v>45</v>
+        <v>44</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>74</v>
+      </c>
+      <c r="B10" t="s">
+        <v>42</v>
+      </c>
+      <c r="C10" t="s">
+        <v>44</v>
       </c>
     </row>
   </sheetData>
@@ -869,10 +892,10 @@
   <sheetData>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C2" t="s">
         <v>4</v>
@@ -880,7 +903,7 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B3" t="s">
         <v>2</v>
@@ -891,10 +914,10 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C4" t="s">
         <v>5</v>
@@ -902,10 +925,10 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C5" t="s">
         <v>5</v>
@@ -913,10 +936,10 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C6" t="s">
         <v>5</v>
@@ -924,18 +947,18 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="B7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C7" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="B8" t="s">
         <v>8</v>
@@ -946,35 +969,35 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="B9" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C9" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="B10" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C10" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="B11" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C11" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
   </sheetData>
@@ -997,7 +1020,7 @@
   <sheetData>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B2" t="s">
         <v>10</v>
@@ -1008,7 +1031,7 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B3" t="s">
         <v>2</v>
@@ -1019,21 +1042,21 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="B4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C5" t="s">
         <v>5</v>
@@ -1041,7 +1064,7 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B6" t="s">
         <v>8</v>
@@ -1052,21 +1075,21 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B7" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C7" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B8" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C8" t="s">
         <v>5</v>
@@ -1074,7 +1097,7 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="B9" t="s">
         <v>8</v>
@@ -1085,24 +1108,24 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="B10" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C10" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="B11" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C11" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
   </sheetData>
@@ -1124,7 +1147,7 @@
         <v>101</v>
       </c>
       <c r="B2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -1132,7 +1155,7 @@
         <v>102</v>
       </c>
       <c r="B3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -1140,7 +1163,7 @@
         <v>103</v>
       </c>
       <c r="B4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -1148,7 +1171,7 @@
         <v>104</v>
       </c>
       <c r="B5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
   </sheetData>
@@ -1170,7 +1193,7 @@
         <v>201</v>
       </c>
       <c r="B2" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -1178,7 +1201,7 @@
         <v>202</v>
       </c>
       <c r="B3" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -1186,7 +1209,7 @@
         <v>203</v>
       </c>
       <c r="B4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -1194,7 +1217,7 @@
         <v>204</v>
       </c>
       <c r="B5" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
     </row>
   </sheetData>
@@ -1216,7 +1239,7 @@
         <v>301</v>
       </c>
       <c r="B2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -1224,7 +1247,7 @@
         <v>302</v>
       </c>
       <c r="B3" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -1232,7 +1255,7 @@
         <v>303</v>
       </c>
       <c r="B4" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -1240,7 +1263,7 @@
         <v>304</v>
       </c>
       <c r="B5" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
     </row>
   </sheetData>
@@ -1265,7 +1288,7 @@
         <v>401</v>
       </c>
       <c r="B2" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -1273,7 +1296,7 @@
         <v>402</v>
       </c>
       <c r="B3" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -1281,7 +1304,7 @@
         <v>403</v>
       </c>
       <c r="B4" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -1289,7 +1312,7 @@
         <v>404</v>
       </c>
       <c r="B5" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -1297,7 +1320,7 @@
         <v>405</v>
       </c>
       <c r="B6" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -1305,7 +1328,7 @@
         <v>406</v>
       </c>
       <c r="B7" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -1313,7 +1336,7 @@
         <v>407</v>
       </c>
       <c r="B8" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -1321,7 +1344,7 @@
         <v>408</v>
       </c>
       <c r="B9" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
@@ -1329,7 +1352,7 @@
         <v>409</v>
       </c>
       <c r="B10" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
@@ -1337,7 +1360,7 @@
         <v>410</v>
       </c>
       <c r="B11" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
     </row>
   </sheetData>
@@ -1357,7 +1380,7 @@
   <sheetData>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="B2" t="s">
         <v>8</v>
@@ -1368,10 +1391,10 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="B3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C3" t="s">
         <v>5</v>
@@ -1379,10 +1402,10 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="B4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C4" t="s">
         <v>5</v>
@@ -1390,10 +1413,10 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="B5" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C5" t="s">
         <v>5</v>
@@ -1401,7 +1424,7 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="B6" t="s">
         <v>3</v>
@@ -1412,7 +1435,7 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>85</v>
+        <v>99</v>
       </c>
       <c r="B7" t="s">
         <v>2</v>
@@ -1439,7 +1462,7 @@
   <sheetData>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="B2" t="s">
         <v>8</v>
@@ -1450,10 +1473,10 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="B3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C3" t="s">
         <v>5</v>
@@ -1461,7 +1484,7 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="B4" t="s">
         <v>3</v>
@@ -1472,7 +1495,7 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="B5" t="s">
         <v>3</v>
@@ -1483,10 +1506,10 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="B6" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="C6" t="s">
         <v>5</v>
@@ -1520,10 +1543,10 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="B3" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="C3" t="s">
         <v>5</v>
@@ -1534,7 +1557,7 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B4" t="s">
         <v>3</v>
@@ -1545,13 +1568,13 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>21</v>
+        <v>100</v>
       </c>
       <c r="B5" t="s">
         <v>11</v>
       </c>
       <c r="C5" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
@@ -1574,7 +1597,7 @@
   <sheetData>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B2" t="s">
         <v>10</v>
@@ -1585,7 +1608,7 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B3" t="s">
         <v>0</v>
@@ -1596,7 +1619,7 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B4" t="s">
         <v>0</v>
@@ -1607,7 +1630,7 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B5" t="s">
         <v>2</v>
@@ -1615,7 +1638,7 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B6" t="s">
         <v>3</v>
@@ -1623,7 +1646,7 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B7" t="s">
         <v>9</v>
@@ -1634,7 +1657,7 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B8" t="s">
         <v>3</v>
@@ -1642,7 +1665,7 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>59</v>
+        <v>101</v>
       </c>
       <c r="B9" t="s">
         <v>11</v>
@@ -1650,7 +1673,7 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B10" t="s">
         <v>3</v>
@@ -1658,7 +1681,7 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>60</v>
+        <v>102</v>
       </c>
       <c r="B11" t="s">
         <v>11</v>
@@ -1677,10 +1700,10 @@
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B13" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C13" t="s">
         <v>5</v>
@@ -1688,7 +1711,7 @@
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="B14" t="s">
         <v>8</v>
@@ -1726,7 +1749,7 @@
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B18" t="s">
         <v>1</v>

</xml_diff>

<commit_message>
Change appointment ID to String and update implementation
</commit_message>
<xml_diff>
--- a/src/main/resources/data/DB.xlsx
+++ b/src/main/resources/data/DB.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4a765bfb693053ce/Desktop/SecurePrints/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="650" documentId="13_ncr:1_{1D354D38-737B-4D3A-A9B1-62F2684C3BE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9A296265-B01A-4AD2-A733-A12C41D6CCDF}"/>
+  <xr:revisionPtr revIDLastSave="673" documentId="13_ncr:1_{1D354D38-737B-4D3A-A9B1-62F2684C3BE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{61EF1859-1941-47F1-AE54-C26B1E8BD0F1}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="810" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="810" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ServiceType" sheetId="5" r:id="rId1"/>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="203" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="104">
   <si>
     <t>varchar(30)</t>
   </si>
@@ -358,7 +358,7 @@
     <t>fbi_rsn_desc</t>
   </si>
   <si>
-    <t>bci_amt</t>
+    <t>bill_amt</t>
   </si>
 </sst>
 </file>
@@ -814,7 +814,7 @@
         <v>22</v>
       </c>
       <c r="C5" t="s">
-        <v>44</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -836,7 +836,7 @@
         <v>8</v>
       </c>
       <c r="C7" t="s">
-        <v>5</v>
+        <v>44</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -1587,7 +1587,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26C3B050-11F0-4CD1-8817-8144CCC481DE}">
-  <dimension ref="A2:C18"/>
+  <dimension ref="A2:C17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.28515625" customWidth="1"/>
@@ -1600,7 +1600,7 @@
         <v>29</v>
       </c>
       <c r="B2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C2" t="s">
         <v>4</v>
@@ -1635,6 +1635,9 @@
       <c r="B5" t="s">
         <v>2</v>
       </c>
+      <c r="C5" t="s">
+        <v>44</v>
+      </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
@@ -1643,6 +1646,9 @@
       <c r="B6" t="s">
         <v>3</v>
       </c>
+      <c r="C6" t="s">
+        <v>44</v>
+      </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
@@ -1662,6 +1668,9 @@
       <c r="B8" t="s">
         <v>3</v>
       </c>
+      <c r="C8" t="s">
+        <v>44</v>
+      </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
@@ -1670,6 +1679,9 @@
       <c r="B9" t="s">
         <v>11</v>
       </c>
+      <c r="C9" t="s">
+        <v>44</v>
+      </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
@@ -1678,6 +1690,9 @@
       <c r="B10" t="s">
         <v>3</v>
       </c>
+      <c r="C10" t="s">
+        <v>44</v>
+      </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
@@ -1686,6 +1701,9 @@
       <c r="B11" t="s">
         <v>11</v>
       </c>
+      <c r="C11" t="s">
+        <v>44</v>
+      </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
@@ -1700,10 +1718,10 @@
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>28</v>
+        <v>58</v>
       </c>
       <c r="B13" t="s">
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="C13" t="s">
         <v>5</v>
@@ -1711,10 +1729,10 @@
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>58</v>
+        <v>12</v>
       </c>
       <c r="B14" t="s">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="C14" t="s">
         <v>5</v>
@@ -1722,37 +1740,35 @@
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B15" t="s">
         <v>1</v>
       </c>
       <c r="C15" t="s">
-        <v>5</v>
+        <v>44</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B16" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C16" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>14</v>
+        <v>36</v>
       </c>
       <c r="B17" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>36</v>
-      </c>
-      <c r="B18" t="s">
-        <v>1</v>
+      <c r="C17" t="s">
+        <v>44</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add cleanup service and generate expense type list
</commit_message>
<xml_diff>
--- a/src/main/resources/data/DB.xlsx
+++ b/src/main/resources/data/DB.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4a765bfb693053ce/Desktop/SecurePrints/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="673" documentId="13_ncr:1_{1D354D38-737B-4D3A-A9B1-62F2684C3BE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{61EF1859-1941-47F1-AE54-C26B1E8BD0F1}"/>
+  <xr:revisionPtr revIDLastSave="875" documentId="13_ncr:1_{1D354D38-737B-4D3A-A9B1-62F2684C3BE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FFA78FBD-CA7F-4760-B1EB-1A6F4ADF864B}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="810" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="810" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ServiceType" sheetId="5" r:id="rId1"/>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="271" uniqueCount="165">
   <si>
     <t>varchar(30)</t>
   </si>
@@ -214,15 +214,9 @@
     <t>exp_ref_dt</t>
   </si>
   <si>
-    <t>exp_type</t>
-  </si>
-  <si>
     <t>varchar(100)</t>
   </si>
   <si>
-    <t>Rent</t>
-  </si>
-  <si>
     <t>appt_sts_code</t>
   </si>
   <si>
@@ -241,27 +235,12 @@
     <t>exp_doc_file</t>
   </si>
   <si>
-    <t>Tax</t>
-  </si>
-  <si>
     <t>Insurance</t>
   </si>
   <si>
     <t>Utilities</t>
   </si>
   <si>
-    <t>Interest</t>
-  </si>
-  <si>
-    <t>Marketing/Advertising</t>
-  </si>
-  <si>
-    <t>Capital Expenditure</t>
-  </si>
-  <si>
-    <t>Wage/Salary/Benefit</t>
-  </si>
-  <si>
     <t>Miscellaneous</t>
   </si>
   <si>
@@ -283,12 +262,6 @@
     <t>exp_rcncl_dt</t>
   </si>
   <si>
-    <t>License</t>
-  </si>
-  <si>
-    <t>Other</t>
-  </si>
-  <si>
     <t>com_name</t>
   </si>
   <si>
@@ -358,7 +331,219 @@
     <t>fbi_rsn_desc</t>
   </si>
   <si>
-    <t>bill_amt</t>
+    <t>bci_amt</t>
+  </si>
+  <si>
+    <t>Check</t>
+  </si>
+  <si>
+    <t>DD</t>
+  </si>
+  <si>
+    <t>Rent or Lease</t>
+  </si>
+  <si>
+    <t>Office, equipment, or vehicle rentals</t>
+  </si>
+  <si>
+    <t>Electricity, water, gas, internet, phone</t>
+  </si>
+  <si>
+    <t>Salaries and Wages</t>
+  </si>
+  <si>
+    <t>Employee compensation</t>
+  </si>
+  <si>
+    <t>Employee Benefits</t>
+  </si>
+  <si>
+    <t>Health insurance, retirement contributions</t>
+  </si>
+  <si>
+    <t>Payroll Taxes</t>
+  </si>
+  <si>
+    <t>Employer-paid taxes like Social Security, Medicare</t>
+  </si>
+  <si>
+    <t>Office Supplies</t>
+  </si>
+  <si>
+    <t>Paper, pens, printer ink, etc</t>
+  </si>
+  <si>
+    <t>Postage and Shipping</t>
+  </si>
+  <si>
+    <t>Mailing or courier services</t>
+  </si>
+  <si>
+    <t>Maintenance and Repairs</t>
+  </si>
+  <si>
+    <t>For office or equipment upkeep</t>
+  </si>
+  <si>
+    <t>Professional Services</t>
+  </si>
+  <si>
+    <t>Legal, accounting, consulting fees</t>
+  </si>
+  <si>
+    <t>Operating Expenses</t>
+  </si>
+  <si>
+    <t>Advertising and Marketing</t>
+  </si>
+  <si>
+    <t>Online ads, billboards, flyers</t>
+  </si>
+  <si>
+    <t>Travel and Meals</t>
+  </si>
+  <si>
+    <t>Business travel, meals with clients</t>
+  </si>
+  <si>
+    <t>Liability, property, workers’ compensation</t>
+  </si>
+  <si>
+    <t>Merchant or transaction fees</t>
+  </si>
+  <si>
+    <t>Software Subscriptions</t>
+  </si>
+  <si>
+    <t>SaaS tools, CRMs, accounting software</t>
+  </si>
+  <si>
+    <t>Licenses and Permits</t>
+  </si>
+  <si>
+    <t>Required by local or federal laws</t>
+  </si>
+  <si>
+    <t>Training and Education</t>
+  </si>
+  <si>
+    <t>Courses, seminars, certifications</t>
+  </si>
+  <si>
+    <t>Dues and Subscriptions</t>
+  </si>
+  <si>
+    <t>Industry memberships, publications</t>
+  </si>
+  <si>
+    <t>Vehicle and Transportation Expenses</t>
+  </si>
+  <si>
+    <t>Fuel and Mileage</t>
+  </si>
+  <si>
+    <t>Vehicle Maintenance and Repairs</t>
+  </si>
+  <si>
+    <t>Vehicle Lease or Depreciation</t>
+  </si>
+  <si>
+    <t>Parking and Tolls</t>
+  </si>
+  <si>
+    <t>Financial Expenses</t>
+  </si>
+  <si>
+    <t>Interest Expense</t>
+  </si>
+  <si>
+    <t>On loans or credit cards</t>
+  </si>
+  <si>
+    <t>Bad Debts</t>
+  </si>
+  <si>
+    <t>Uncollectible customer invoices</t>
+  </si>
+  <si>
+    <t>Gifts</t>
+  </si>
+  <si>
+    <t>Charitable Contributions</t>
+  </si>
+  <si>
+    <t>Penalties and Fines</t>
+  </si>
+  <si>
+    <t>Within allowable business limits</t>
+  </si>
+  <si>
+    <t>If tax-deductible</t>
+  </si>
+  <si>
+    <t>Not usually tax-deductible, but recorded</t>
+  </si>
+  <si>
+    <t>Depreciation</t>
+  </si>
+  <si>
+    <t>Amortization</t>
+  </si>
+  <si>
+    <t>Tangible assets (physical items: Buildings, machinery, vehicles, computers)</t>
+  </si>
+  <si>
+    <t>You buy a $10,000 computer for your business, expected to last 5 years.
+→ You record $2,000 per year as depreciation expense.</t>
+  </si>
+  <si>
+    <t>You acquire a software license for $15,000, valid for 3 years.
+→ You record $5,000 per year as amortization expense.</t>
+  </si>
+  <si>
+    <t>Non-Operating Expenses</t>
+  </si>
+  <si>
+    <t>Cost of borrowing money (loans, credit lines, bonds)</t>
+  </si>
+  <si>
+    <t>Income Tax Expense</t>
+  </si>
+  <si>
+    <t>Taxes paid on business profits</t>
+  </si>
+  <si>
+    <t>Loss on Sale of Assets</t>
+  </si>
+  <si>
+    <t>When a business sells an asset for less than its book value</t>
+  </si>
+  <si>
+    <t>Selling a machine for $5,000 that was on the books for $7,000 → $2,000 loss</t>
+  </si>
+  <si>
+    <t>Restructuring Costs</t>
+  </si>
+  <si>
+    <t>Expenses from reorganizing the business (layoffs, plant closures, etc.)</t>
+  </si>
+  <si>
+    <t>Write-offs of Uncollectible Debts (Bad Debt Expense)</t>
+  </si>
+  <si>
+    <t>When a customer invoice is deemed non-recoverable</t>
+  </si>
+  <si>
+    <t>exp_type_code</t>
+  </si>
+  <si>
+    <t>Selling and Administrative Expenses</t>
+  </si>
+  <si>
+    <t>Bank Fees and Credit Card Processing</t>
+  </si>
+  <si>
+    <t>Intangible assets (non-physical items: Patents, copyrights, trademarks, software licenses, goodwill)</t>
   </si>
 </sst>
 </file>
@@ -368,7 +553,7 @@
   <numFmts count="1">
     <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -395,6 +580,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -417,13 +610,23 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Currency" xfId="1" builtinId="4"/>
@@ -440,6 +643,55 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>48</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>1762828</xdr:colOff>
+      <xdr:row>80</xdr:row>
+      <xdr:rowOff>115167</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{ED12F31F-2474-ABD5-2E0D-9D0FE385E825}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="609600" y="12001500"/>
+          <a:ext cx="5039428" cy="6211167"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
@@ -808,7 +1060,7 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>103</v>
+        <v>94</v>
       </c>
       <c r="B5" t="s">
         <v>22</v>
@@ -819,7 +1071,7 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>92</v>
+        <v>83</v>
       </c>
       <c r="B6" t="s">
         <v>8</v>
@@ -830,7 +1082,7 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>91</v>
+        <v>82</v>
       </c>
       <c r="B7" t="s">
         <v>8</v>
@@ -852,10 +1104,10 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="B9" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C9" t="s">
         <v>44</v>
@@ -863,7 +1115,7 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>74</v>
+        <v>67</v>
       </c>
       <c r="B10" t="s">
         <v>42</v>
@@ -947,7 +1199,7 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>73</v>
+        <v>66</v>
       </c>
       <c r="B7" t="s">
         <v>40</v>
@@ -958,7 +1210,7 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>97</v>
+        <v>88</v>
       </c>
       <c r="B8" t="s">
         <v>8</v>
@@ -969,7 +1221,7 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>96</v>
+        <v>87</v>
       </c>
       <c r="B9" t="s">
         <v>42</v>
@@ -980,10 +1232,10 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>75</v>
+        <v>68</v>
       </c>
       <c r="B10" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C10" t="s">
         <v>44</v>
@@ -991,7 +1243,7 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>76</v>
+        <v>69</v>
       </c>
       <c r="B11" t="s">
         <v>42</v>
@@ -1042,7 +1294,7 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="B4" t="s">
         <v>41</v>
@@ -1064,7 +1316,7 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>55</v>
+        <v>161</v>
       </c>
       <c r="B6" t="s">
         <v>8</v>
@@ -1078,7 +1330,7 @@
         <v>51</v>
       </c>
       <c r="B7" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C7" t="s">
         <v>44</v>
@@ -1097,7 +1349,7 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>98</v>
+        <v>89</v>
       </c>
       <c r="B9" t="s">
         <v>8</v>
@@ -1108,7 +1360,7 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="B10" t="s">
         <v>40</v>
@@ -1119,7 +1371,7 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>77</v>
+        <v>70</v>
       </c>
       <c r="B11" t="s">
         <v>42</v>
@@ -1193,7 +1445,7 @@
         <v>201</v>
       </c>
       <c r="B2" t="s">
-        <v>95</v>
+        <v>86</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -1201,7 +1453,7 @@
         <v>202</v>
       </c>
       <c r="B3" t="s">
-        <v>93</v>
+        <v>84</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -1217,7 +1469,7 @@
         <v>204</v>
       </c>
       <c r="B5" t="s">
-        <v>94</v>
+        <v>85</v>
       </c>
     </row>
   </sheetData>
@@ -1227,7 +1479,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CDB63C17-C30B-42C8-BC51-3A749A87B21E}">
-  <dimension ref="A2:B5"/>
+  <dimension ref="A2:B6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="2"/>
@@ -1255,7 +1507,7 @@
         <v>303</v>
       </c>
       <c r="B4" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -1263,7 +1515,15 @@
         <v>304</v>
       </c>
       <c r="B5" t="s">
-        <v>79</v>
+        <v>95</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" s="2">
+        <v>305</v>
+      </c>
+      <c r="B6" t="s">
+        <v>96</v>
       </c>
     </row>
   </sheetData>
@@ -1276,95 +1536,409 @@
   <sheetPr>
     <tabColor theme="7"/>
   </sheetPr>
-  <dimension ref="A2:B11"/>
+  <dimension ref="A2:D45"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="2"/>
-    <col min="2" max="2" width="25.5703125" customWidth="1"/>
+    <col min="2" max="2" width="49.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="64.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="67.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="2">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B2" s="4" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" s="2">
         <v>401</v>
       </c>
-      <c r="B2" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="2">
+      <c r="B3" t="s">
+        <v>97</v>
+      </c>
+      <c r="C3" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" s="2">
         <v>402</v>
       </c>
-      <c r="B3" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="2">
+      <c r="B4" t="s">
+        <v>63</v>
+      </c>
+      <c r="C4" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" s="2">
         <v>403</v>
       </c>
-      <c r="B4" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="2">
+      <c r="B5" t="s">
+        <v>100</v>
+      </c>
+      <c r="C5" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" s="2">
         <v>404</v>
       </c>
-      <c r="B5" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="2">
+      <c r="B6" t="s">
+        <v>102</v>
+      </c>
+      <c r="C6" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" s="2">
         <v>405</v>
       </c>
-      <c r="B6" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" s="2">
+      <c r="B7" t="s">
+        <v>104</v>
+      </c>
+      <c r="C7" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" s="2">
         <v>406</v>
       </c>
-      <c r="B7" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" s="2">
+      <c r="B8" t="s">
+        <v>106</v>
+      </c>
+      <c r="C8" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" s="2">
         <v>407</v>
       </c>
-      <c r="B8" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" s="2">
+      <c r="B9" t="s">
+        <v>108</v>
+      </c>
+      <c r="C9" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" s="2">
         <v>408</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B10" t="s">
+        <v>110</v>
+      </c>
+      <c r="C10" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" s="2">
+        <v>409</v>
+      </c>
+      <c r="B11" t="s">
+        <v>112</v>
+      </c>
+      <c r="C11" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B13" s="4" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14" s="2">
+        <v>501</v>
+      </c>
+      <c r="B14" t="s">
+        <v>135</v>
+      </c>
+      <c r="C14" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15" s="2">
+        <v>502</v>
+      </c>
+      <c r="B15" t="s">
+        <v>152</v>
+      </c>
+      <c r="C15" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" s="2">
+        <v>503</v>
+      </c>
+      <c r="B16" t="s">
+        <v>154</v>
+      </c>
+      <c r="C16" t="s">
+        <v>155</v>
+      </c>
+      <c r="D16" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17" s="2">
+        <v>504</v>
+      </c>
+      <c r="B17" t="s">
+        <v>157</v>
+      </c>
+      <c r="C17" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18" s="2">
+        <v>505</v>
+      </c>
+      <c r="B18" t="s">
+        <v>159</v>
+      </c>
+      <c r="C18" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B20" s="4" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A21" s="2">
+        <v>601</v>
+      </c>
+      <c r="B21" t="s">
+        <v>115</v>
+      </c>
+      <c r="C21" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A22" s="2">
+        <v>602</v>
+      </c>
+      <c r="B22" t="s">
+        <v>117</v>
+      </c>
+      <c r="C22" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A23" s="2">
+        <v>603</v>
+      </c>
+      <c r="B23" t="s">
+        <v>62</v>
+      </c>
+      <c r="C23" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A24" s="2">
+        <v>604</v>
+      </c>
+      <c r="B24" t="s">
+        <v>163</v>
+      </c>
+      <c r="C24" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A25" s="2">
+        <v>605</v>
+      </c>
+      <c r="B25" t="s">
+        <v>121</v>
+      </c>
+      <c r="C25" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A26" s="2">
+        <v>606</v>
+      </c>
+      <c r="B26" t="s">
+        <v>123</v>
+      </c>
+      <c r="C26" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A27" s="2">
+        <v>607</v>
+      </c>
+      <c r="B27" t="s">
+        <v>125</v>
+      </c>
+      <c r="C27" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A28" s="2">
+        <v>608</v>
+      </c>
+      <c r="B28" t="s">
+        <v>127</v>
+      </c>
+      <c r="C28" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B30" s="4" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A31" s="2">
+        <v>701</v>
+      </c>
+      <c r="B31" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A32" s="2">
+        <v>702</v>
+      </c>
+      <c r="B32" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A33" s="2">
+        <v>703</v>
+      </c>
+      <c r="B33" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A34" s="2">
+        <v>704</v>
+      </c>
+      <c r="B34" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B36" s="4" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A37" s="2">
+        <v>801</v>
+      </c>
+      <c r="B37" t="s">
+        <v>135</v>
+      </c>
+      <c r="C37" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A38" s="2">
+        <v>802</v>
+      </c>
+      <c r="B38" t="s">
+        <v>137</v>
+      </c>
+      <c r="C38" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A39" s="7">
+        <v>803</v>
+      </c>
+      <c r="B39" s="6" t="s">
+        <v>145</v>
+      </c>
+      <c r="C39" s="5" t="s">
+        <v>147</v>
+      </c>
+      <c r="D39" s="5" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A40" s="7">
+        <v>804</v>
+      </c>
+      <c r="B40" s="6" t="s">
+        <v>146</v>
+      </c>
+      <c r="C40" s="5" t="s">
+        <v>164</v>
+      </c>
+      <c r="D40" s="5" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B42" s="4" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10" s="2">
-        <v>409</v>
-      </c>
-      <c r="B10" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A11" s="2">
-        <v>410</v>
-      </c>
-      <c r="B11" t="s">
-        <v>71</v>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A43" s="2">
+        <v>901</v>
+      </c>
+      <c r="B43" t="s">
+        <v>139</v>
+      </c>
+      <c r="C43" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A44" s="2">
+        <v>902</v>
+      </c>
+      <c r="B44" t="s">
+        <v>140</v>
+      </c>
+      <c r="C44" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A45" s="2">
+        <v>903</v>
+      </c>
+      <c r="B45" t="s">
+        <v>141</v>
+      </c>
+      <c r="C45" t="s">
+        <v>144</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -1380,7 +1954,7 @@
   <sheetData>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>82</v>
+        <v>73</v>
       </c>
       <c r="B2" t="s">
         <v>8</v>
@@ -1391,7 +1965,7 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>80</v>
+        <v>71</v>
       </c>
       <c r="B3" t="s">
         <v>40</v>
@@ -1402,10 +1976,10 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="B4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C4" t="s">
         <v>5</v>
@@ -1413,10 +1987,10 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="B5" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C5" t="s">
         <v>5</v>
@@ -1424,7 +1998,7 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>81</v>
+        <v>72</v>
       </c>
       <c r="B6" t="s">
         <v>3</v>
@@ -1435,7 +2009,7 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>99</v>
+        <v>90</v>
       </c>
       <c r="B7" t="s">
         <v>2</v>
@@ -1462,7 +2036,7 @@
   <sheetData>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>83</v>
+        <v>74</v>
       </c>
       <c r="B2" t="s">
         <v>8</v>
@@ -1473,7 +2047,7 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>84</v>
+        <v>75</v>
       </c>
       <c r="B3" t="s">
         <v>40</v>
@@ -1484,7 +2058,7 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>85</v>
+        <v>76</v>
       </c>
       <c r="B4" t="s">
         <v>3</v>
@@ -1495,7 +2069,7 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>86</v>
+        <v>77</v>
       </c>
       <c r="B5" t="s">
         <v>3</v>
@@ -1506,10 +2080,10 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="B6" t="s">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="C6" t="s">
         <v>5</v>
@@ -1543,10 +2117,10 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="B3" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="C3" t="s">
         <v>5</v>
@@ -1568,7 +2142,7 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>100</v>
+        <v>91</v>
       </c>
       <c r="B5" t="s">
         <v>11</v>
@@ -1674,7 +2248,7 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>101</v>
+        <v>92</v>
       </c>
       <c r="B9" t="s">
         <v>11</v>
@@ -1696,7 +2270,7 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>102</v>
+        <v>93</v>
       </c>
       <c r="B11" t="s">
         <v>11</v>
@@ -1718,7 +2292,7 @@
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B13" t="s">
         <v>8</v>

</xml_diff>

<commit_message>
Add expense and invoice entities, repo, service and controller with implement add and view expense
</commit_message>
<xml_diff>
--- a/src/main/resources/data/DB.xlsx
+++ b/src/main/resources/data/DB.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4a765bfb693053ce/Desktop/SecurePrints/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="875" documentId="13_ncr:1_{1D354D38-737B-4D3A-A9B1-62F2684C3BE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FFA78FBD-CA7F-4760-B1EB-1A6F4ADF864B}"/>
+  <xr:revisionPtr revIDLastSave="914" documentId="13_ncr:1_{1D354D38-737B-4D3A-A9B1-62F2684C3BE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0FE8F0E3-27D0-4285-B618-5F7E45602F7E}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="810" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="810" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ServiceType" sheetId="5" r:id="rId1"/>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="271" uniqueCount="165">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="286" uniqueCount="170">
   <si>
     <t>varchar(30)</t>
   </si>
@@ -184,9 +184,6 @@
     <t>Null</t>
   </si>
   <si>
-    <t>inv_clnt_name</t>
-  </si>
-  <si>
     <t>pymt_dt</t>
   </si>
   <si>
@@ -232,9 +229,6 @@
     <t>exp_ref_no</t>
   </si>
   <si>
-    <t>exp_doc_file</t>
-  </si>
-  <si>
     <t>Insurance</t>
   </si>
   <si>
@@ -245,9 +239,6 @@
   </si>
   <si>
     <t>pymt_cmt</t>
-  </si>
-  <si>
-    <t>inv_doc_file</t>
   </si>
   <si>
     <t>pymt_rcncl_dt</t>
@@ -534,9 +525,6 @@
     <t>When a customer invoice is deemed non-recoverable</t>
   </si>
   <si>
-    <t>exp_type_code</t>
-  </si>
-  <si>
     <t>Selling and Administrative Expenses</t>
   </si>
   <si>
@@ -544,6 +532,33 @@
   </si>
   <si>
     <t>Intangible assets (non-physical items: Patents, copyrights, trademarks, software licenses, goodwill)</t>
+  </si>
+  <si>
+    <t>inv_pymt_method_code</t>
+  </si>
+  <si>
+    <t>exp_pymt_dt</t>
+  </si>
+  <si>
+    <t>exp_pymt_method_code</t>
+  </si>
+  <si>
+    <t>inv_payee_name</t>
+  </si>
+  <si>
+    <t>UNIQUE</t>
+  </si>
+  <si>
+    <t>exp_cat_code</t>
+  </si>
+  <si>
+    <t>exp_sub_cat_code</t>
+  </si>
+  <si>
+    <t>exp_doc_file_name</t>
+  </si>
+  <si>
+    <t>inv_doc_file_name</t>
   </si>
 </sst>
 </file>
@@ -1001,7 +1016,7 @@
         <v>20</v>
       </c>
       <c r="B4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C4" s="1">
         <v>68</v>
@@ -1060,7 +1075,7 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="B5" t="s">
         <v>22</v>
@@ -1071,7 +1086,7 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="B6" t="s">
         <v>8</v>
@@ -1082,7 +1097,7 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="B7" t="s">
         <v>8</v>
@@ -1093,7 +1108,7 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B8" t="s">
         <v>42</v>
@@ -1104,10 +1119,10 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B9" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C9" t="s">
         <v>44</v>
@@ -1115,7 +1130,7 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="B10" t="s">
         <v>42</v>
@@ -1131,13 +1146,10 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D7918C8B-2669-416D-A3E8-BF043A7D1DA9}">
-  <sheetPr>
-    <tabColor theme="7"/>
-  </sheetPr>
-  <dimension ref="A2:C11"/>
+  <dimension ref="A2:C12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="20.140625" customWidth="1"/>
+    <col min="1" max="1" width="24.140625" customWidth="1"/>
     <col min="2" max="2" width="14.140625" customWidth="1"/>
     <col min="3" max="3" width="12.42578125" customWidth="1"/>
   </cols>
@@ -1155,7 +1167,7 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>45</v>
+        <v>164</v>
       </c>
       <c r="B3" t="s">
         <v>2</v>
@@ -1199,32 +1211,32 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>66</v>
+        <v>85</v>
       </c>
       <c r="B7" t="s">
-        <v>40</v>
+        <v>8</v>
       </c>
       <c r="C7" t="s">
-        <v>44</v>
+        <v>5</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="B8" t="s">
-        <v>8</v>
+        <v>42</v>
       </c>
       <c r="C8" t="s">
-        <v>5</v>
+        <v>44</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>87</v>
+        <v>161</v>
       </c>
       <c r="B9" t="s">
-        <v>42</v>
+        <v>8</v>
       </c>
       <c r="C9" t="s">
         <v>44</v>
@@ -1232,10 +1244,10 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="B10" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C10" t="s">
         <v>44</v>
@@ -1243,12 +1255,23 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>69</v>
+        <v>169</v>
       </c>
       <c r="B11" t="s">
+        <v>40</v>
+      </c>
+      <c r="C11" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>66</v>
+      </c>
+      <c r="B12" t="s">
         <v>42</v>
       </c>
-      <c r="C11" t="s">
+      <c r="C12" t="s">
         <v>44</v>
       </c>
     </row>
@@ -1259,20 +1282,18 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5759F7E4-D816-4B52-AE2B-CD03ABF39BDB}">
-  <sheetPr>
-    <tabColor theme="7"/>
-  </sheetPr>
-  <dimension ref="A2:C11"/>
+  <dimension ref="A2:D14"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="20.85546875" customWidth="1"/>
+    <col min="1" max="1" width="25.42578125" customWidth="1"/>
     <col min="2" max="2" width="12.5703125" customWidth="1"/>
     <col min="3" max="3" width="12.85546875" customWidth="1"/>
+    <col min="4" max="4" width="14.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B2" t="s">
         <v>10</v>
@@ -1281,9 +1302,9 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B3" t="s">
         <v>2</v>
@@ -1292,20 +1313,23 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B4" t="s">
         <v>41</v>
       </c>
       <c r="C4" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+      <c r="D4" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B5" t="s">
         <v>42</v>
@@ -1314,9 +1338,9 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>161</v>
+        <v>166</v>
       </c>
       <c r="B6" t="s">
         <v>8</v>
@@ -1325,58 +1349,91 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>51</v>
+        <v>167</v>
       </c>
       <c r="B7" t="s">
-        <v>55</v>
+        <v>8</v>
       </c>
       <c r="C7" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>50</v>
+      </c>
+      <c r="B8" t="s">
+        <v>54</v>
+      </c>
+      <c r="C8" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>53</v>
-      </c>
-      <c r="B8" t="s">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>52</v>
+      </c>
+      <c r="B9" t="s">
         <v>22</v>
       </c>
-      <c r="C8" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>89</v>
-      </c>
-      <c r="B9" t="s">
+      <c r="C9" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>86</v>
+      </c>
+      <c r="B10" t="s">
         <v>8</v>
       </c>
-      <c r="C9" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>61</v>
-      </c>
-      <c r="B10" t="s">
-        <v>40</v>
-      </c>
       <c r="C10" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>70</v>
+        <v>162</v>
       </c>
       <c r="B11" t="s">
         <v>42</v>
       </c>
       <c r="C11" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>163</v>
+      </c>
+      <c r="B12" t="s">
+        <v>8</v>
+      </c>
+      <c r="C12" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>168</v>
+      </c>
+      <c r="B13" t="s">
+        <v>40</v>
+      </c>
+      <c r="C13" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>67</v>
+      </c>
+      <c r="B14" t="s">
+        <v>42</v>
+      </c>
+      <c r="C14" t="s">
         <v>44</v>
       </c>
     </row>
@@ -1445,7 +1502,7 @@
         <v>201</v>
       </c>
       <c r="B2" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -1453,7 +1510,7 @@
         <v>202</v>
       </c>
       <c r="B3" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -1469,7 +1526,7 @@
         <v>204</v>
       </c>
       <c r="B5" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
     </row>
   </sheetData>
@@ -1491,7 +1548,7 @@
         <v>301</v>
       </c>
       <c r="B2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -1499,7 +1556,7 @@
         <v>302</v>
       </c>
       <c r="B3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -1507,7 +1564,7 @@
         <v>303</v>
       </c>
       <c r="B4" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -1515,7 +1572,7 @@
         <v>304</v>
       </c>
       <c r="B5" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -1523,7 +1580,7 @@
         <v>305</v>
       </c>
       <c r="B6" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
     </row>
   </sheetData>
@@ -1533,9 +1590,6 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B7D22FEC-2373-4675-B83F-6DA956326EDE}">
-  <sheetPr>
-    <tabColor theme="7"/>
-  </sheetPr>
   <dimension ref="A2:D45"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1547,7 +1601,7 @@
   <sheetData>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B2" s="4" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -1555,10 +1609,10 @@
         <v>401</v>
       </c>
       <c r="B3" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="C3" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -1566,10 +1620,10 @@
         <v>402</v>
       </c>
       <c r="B4" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="C4" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
@@ -1577,10 +1631,10 @@
         <v>403</v>
       </c>
       <c r="B5" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="C5" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -1588,10 +1642,10 @@
         <v>404</v>
       </c>
       <c r="B6" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="C6" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
@@ -1599,10 +1653,10 @@
         <v>405</v>
       </c>
       <c r="B7" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="C7" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
@@ -1610,10 +1664,10 @@
         <v>406</v>
       </c>
       <c r="B8" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="C8" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
@@ -1621,10 +1675,10 @@
         <v>407</v>
       </c>
       <c r="B9" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="C9" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
@@ -1632,10 +1686,10 @@
         <v>408</v>
       </c>
       <c r="B10" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="C10" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
@@ -1643,15 +1697,15 @@
         <v>409</v>
       </c>
       <c r="B11" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="C11" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B13" s="4" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
@@ -1659,10 +1713,10 @@
         <v>501</v>
       </c>
       <c r="B14" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="C14" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
@@ -1670,10 +1724,10 @@
         <v>502</v>
       </c>
       <c r="B15" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="C15" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
@@ -1681,13 +1735,13 @@
         <v>503</v>
       </c>
       <c r="B16" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="C16" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="D16" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
@@ -1695,10 +1749,10 @@
         <v>504</v>
       </c>
       <c r="B17" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="C17" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
@@ -1706,15 +1760,15 @@
         <v>505</v>
       </c>
       <c r="B18" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="C18" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B20" s="4" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
@@ -1722,10 +1776,10 @@
         <v>601</v>
       </c>
       <c r="B21" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="C21" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
@@ -1733,10 +1787,10 @@
         <v>602</v>
       </c>
       <c r="B22" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="C22" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
@@ -1744,10 +1798,10 @@
         <v>603</v>
       </c>
       <c r="B23" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C23" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
@@ -1755,10 +1809,10 @@
         <v>604</v>
       </c>
       <c r="B24" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="C24" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
@@ -1766,10 +1820,10 @@
         <v>605</v>
       </c>
       <c r="B25" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="C25" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
@@ -1777,10 +1831,10 @@
         <v>606</v>
       </c>
       <c r="B26" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="C26" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
@@ -1788,10 +1842,10 @@
         <v>607</v>
       </c>
       <c r="B27" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="C27" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
@@ -1799,15 +1853,15 @@
         <v>608</v>
       </c>
       <c r="B28" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="C28" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B30" s="4" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
@@ -1815,7 +1869,7 @@
         <v>701</v>
       </c>
       <c r="B31" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
@@ -1823,7 +1877,7 @@
         <v>702</v>
       </c>
       <c r="B32" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
@@ -1831,7 +1885,7 @@
         <v>703</v>
       </c>
       <c r="B33" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
@@ -1839,12 +1893,12 @@
         <v>704</v>
       </c>
       <c r="B34" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B36" s="4" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
@@ -1852,10 +1906,10 @@
         <v>801</v>
       </c>
       <c r="B37" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="C37" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
@@ -1863,10 +1917,10 @@
         <v>802</v>
       </c>
       <c r="B38" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="C38" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
     </row>
     <row r="39" spans="1:4" ht="30" x14ac:dyDescent="0.25">
@@ -1874,13 +1928,13 @@
         <v>803</v>
       </c>
       <c r="B39" s="6" t="s">
+        <v>142</v>
+      </c>
+      <c r="C39" s="5" t="s">
+        <v>144</v>
+      </c>
+      <c r="D39" s="5" t="s">
         <v>145</v>
-      </c>
-      <c r="C39" s="5" t="s">
-        <v>147</v>
-      </c>
-      <c r="D39" s="5" t="s">
-        <v>148</v>
       </c>
     </row>
     <row r="40" spans="1:4" ht="30" x14ac:dyDescent="0.25">
@@ -1888,18 +1942,18 @@
         <v>804</v>
       </c>
       <c r="B40" s="6" t="s">
+        <v>143</v>
+      </c>
+      <c r="C40" s="5" t="s">
+        <v>160</v>
+      </c>
+      <c r="D40" s="5" t="s">
         <v>146</v>
-      </c>
-      <c r="C40" s="5" t="s">
-        <v>164</v>
-      </c>
-      <c r="D40" s="5" t="s">
-        <v>149</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B42" s="4" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
@@ -1907,10 +1961,10 @@
         <v>901</v>
       </c>
       <c r="B43" t="s">
+        <v>136</v>
+      </c>
+      <c r="C43" t="s">
         <v>139</v>
-      </c>
-      <c r="C43" t="s">
-        <v>142</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
@@ -1918,10 +1972,10 @@
         <v>902</v>
       </c>
       <c r="B44" t="s">
+        <v>137</v>
+      </c>
+      <c r="C44" t="s">
         <v>140</v>
-      </c>
-      <c r="C44" t="s">
-        <v>143</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
@@ -1929,10 +1983,10 @@
         <v>903</v>
       </c>
       <c r="B45" t="s">
+        <v>138</v>
+      </c>
+      <c r="C45" t="s">
         <v>141</v>
-      </c>
-      <c r="C45" t="s">
-        <v>144</v>
       </c>
     </row>
   </sheetData>
@@ -1944,17 +1998,18 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3A86F615-CD80-437A-AC5A-B0FC5385ACDF}">
-  <dimension ref="A2:C7"/>
+  <dimension ref="A2:D7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.7109375" customWidth="1"/>
     <col min="2" max="2" width="14.28515625" customWidth="1"/>
     <col min="3" max="3" width="13.7109375" customWidth="1"/>
+    <col min="4" max="4" width="14.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="B2" t="s">
         <v>8</v>
@@ -1963,9 +2018,9 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="B3" t="s">
         <v>40</v>
@@ -1973,32 +2028,35 @@
       <c r="C3" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D3" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="B4" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C4" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="B5" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C5" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="B6" t="s">
         <v>3</v>
@@ -2007,9 +2065,9 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="B7" t="s">
         <v>2</v>
@@ -2026,17 +2084,18 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{96185082-E4A1-4DED-800D-93BF3456C969}">
-  <dimension ref="A2:C6"/>
+  <dimension ref="A2:D6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.42578125" customWidth="1"/>
     <col min="2" max="2" width="14.7109375" customWidth="1"/>
     <col min="3" max="3" width="16.5703125" customWidth="1"/>
+    <col min="4" max="4" width="12.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="B2" t="s">
         <v>8</v>
@@ -2045,9 +2104,9 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="B3" t="s">
         <v>40</v>
@@ -2056,9 +2115,9 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="B4" t="s">
         <v>3</v>
@@ -2066,10 +2125,13 @@
       <c r="C4" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D4" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="B5" t="s">
         <v>3</v>
@@ -2078,12 +2140,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="B6" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="C6" t="s">
         <v>5</v>
@@ -2117,10 +2179,10 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>56</v>
+      </c>
+      <c r="B3" t="s">
         <v>57</v>
-      </c>
-      <c r="B3" t="s">
-        <v>58</v>
       </c>
       <c r="C3" t="s">
         <v>5</v>
@@ -2142,7 +2204,7 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="B5" t="s">
         <v>11</v>
@@ -2248,7 +2310,7 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="B9" t="s">
         <v>11</v>
@@ -2270,7 +2332,7 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="B11" t="s">
         <v>11</v>
@@ -2292,7 +2354,7 @@
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B13" t="s">
         <v>8</v>

</xml_diff>

<commit_message>
Add new column to expense and payment tables
</commit_message>
<xml_diff>
--- a/src/main/resources/data/DB.xlsx
+++ b/src/main/resources/data/DB.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4a765bfb693053ce/Desktop/SecurePrints/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="914" documentId="13_ncr:1_{1D354D38-737B-4D3A-A9B1-62F2684C3BE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0FE8F0E3-27D0-4285-B618-5F7E45602F7E}"/>
+  <xr:revisionPtr revIDLastSave="920" documentId="13_ncr:1_{1D354D38-737B-4D3A-A9B1-62F2684C3BE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{48290CC1-59E3-462A-A4DB-4E2178324325}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="810" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="810" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ServiceType" sheetId="5" r:id="rId1"/>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="286" uniqueCount="170">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="292" uniqueCount="172">
   <si>
     <t>varchar(30)</t>
   </si>
@@ -559,6 +559,12 @@
   </si>
   <si>
     <t>inv_doc_file_name</t>
+  </si>
+  <si>
+    <t>exp_updt</t>
+  </si>
+  <si>
+    <t>pymt_updt</t>
   </si>
 </sst>
 </file>
@@ -1032,7 +1038,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{499D205C-AB14-4D61-B52D-6BDE054EBB20}">
-  <dimension ref="A2:C10"/>
+  <dimension ref="A2:C11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20.85546875" customWidth="1"/>
@@ -1137,6 +1143,17 @@
       </c>
       <c r="C10" t="s">
         <v>44</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>171</v>
+      </c>
+      <c r="B11" t="s">
+        <v>76</v>
+      </c>
+      <c r="C11" t="s">
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -1282,7 +1299,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5759F7E4-D816-4B52-AE2B-CD03ABF39BDB}">
-  <dimension ref="A2:D14"/>
+  <dimension ref="A2:D15"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.42578125" customWidth="1"/>
@@ -1435,6 +1452,17 @@
       </c>
       <c r="C14" t="s">
         <v>44</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>170</v>
+      </c>
+      <c r="B15" t="s">
+        <v>76</v>
+      </c>
+      <c r="C15" t="s">
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add appointment payment implementation
</commit_message>
<xml_diff>
--- a/src/main/resources/data/DB.xlsx
+++ b/src/main/resources/data/DB.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4a765bfb693053ce/Desktop/SecurePrints/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="920" documentId="13_ncr:1_{1D354D38-737B-4D3A-A9B1-62F2684C3BE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{48290CC1-59E3-462A-A4DB-4E2178324325}"/>
+  <xr:revisionPtr revIDLastSave="921" documentId="13_ncr:1_{1D354D38-737B-4D3A-A9B1-62F2684C3BE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2735BD37-A862-42A1-9DDD-9BC8E6892557}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="810" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="810" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ServiceType" sheetId="5" r:id="rId1"/>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="292" uniqueCount="172">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="289" uniqueCount="172">
   <si>
     <t>varchar(30)</t>
   </si>
@@ -1038,7 +1038,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{499D205C-AB14-4D61-B52D-6BDE054EBB20}">
-  <dimension ref="A2:C11"/>
+  <dimension ref="A2:C10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20.85546875" customWidth="1"/>
@@ -1059,10 +1059,10 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B3" t="s">
-        <v>9</v>
+        <v>22</v>
       </c>
       <c r="C3" t="s">
         <v>5</v>
@@ -1070,7 +1070,7 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>28</v>
+        <v>91</v>
       </c>
       <c r="B4" t="s">
         <v>22</v>
@@ -1081,10 +1081,10 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>91</v>
+        <v>80</v>
       </c>
       <c r="B5" t="s">
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="C5" t="s">
         <v>5</v>
@@ -1092,43 +1092,43 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B6" t="s">
         <v>8</v>
       </c>
       <c r="C6" t="s">
-        <v>5</v>
+        <v>44</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>79</v>
+        <v>45</v>
       </c>
       <c r="B7" t="s">
-        <v>8</v>
+        <v>42</v>
       </c>
       <c r="C7" t="s">
-        <v>44</v>
+        <v>5</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>45</v>
+        <v>63</v>
       </c>
       <c r="B8" t="s">
-        <v>42</v>
+        <v>54</v>
       </c>
       <c r="C8" t="s">
-        <v>5</v>
+        <v>44</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B9" t="s">
-        <v>54</v>
+        <v>42</v>
       </c>
       <c r="C9" t="s">
         <v>44</v>
@@ -1136,23 +1136,12 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>64</v>
+        <v>171</v>
       </c>
       <c r="B10" t="s">
-        <v>42</v>
+        <v>76</v>
       </c>
       <c r="C10" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>171</v>
-      </c>
-      <c r="B11" t="s">
-        <v>76</v>
-      </c>
-      <c r="C11" t="s">
         <v>5</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Password and DB encryption
</commit_message>
<xml_diff>
--- a/src/main/resources/data/DB.xlsx
+++ b/src/main/resources/data/DB.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4a765bfb693053ce/Desktop/SecurePrints/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="921" documentId="13_ncr:1_{1D354D38-737B-4D3A-A9B1-62F2684C3BE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2735BD37-A862-42A1-9DDD-9BC8E6892557}"/>
+  <xr:revisionPtr revIDLastSave="923" documentId="13_ncr:1_{1D354D38-737B-4D3A-A9B1-62F2684C3BE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1F20B045-936A-4275-82D1-809E8F0FB383}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="810" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="810" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ServiceType" sheetId="5" r:id="rId1"/>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="289" uniqueCount="172">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="289" uniqueCount="173">
   <si>
     <t>varchar(30)</t>
   </si>
@@ -565,6 +565,9 @@
   </si>
   <si>
     <t>pymt_updt</t>
+  </si>
+  <si>
+    <t>text</t>
   </si>
 </sst>
 </file>
@@ -2151,7 +2154,7 @@
         <v>74</v>
       </c>
       <c r="B5" t="s">
-        <v>3</v>
+        <v>172</v>
       </c>
       <c r="C5" t="s">
         <v>5</v>
@@ -2297,7 +2300,7 @@
         <v>26</v>
       </c>
       <c r="B6" t="s">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="C6" t="s">
         <v>44</v>

</xml_diff>

<commit_message>
Change PK of user entity
</commit_message>
<xml_diff>
--- a/src/main/resources/data/DB.xlsx
+++ b/src/main/resources/data/DB.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4a765bfb693053ce/Desktop/SecurePrints/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="923" documentId="13_ncr:1_{1D354D38-737B-4D3A-A9B1-62F2684C3BE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1F20B045-936A-4275-82D1-809E8F0FB383}"/>
+  <xr:revisionPtr revIDLastSave="931" documentId="13_ncr:1_{1D354D38-737B-4D3A-A9B1-62F2684C3BE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{224434E3-24A7-4BFD-9312-C703A323121B}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="810" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="289" uniqueCount="173">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="290" uniqueCount="174">
   <si>
     <t>varchar(30)</t>
   </si>
@@ -568,6 +568,9 @@
   </si>
   <si>
     <t>text</t>
+  </si>
+  <si>
+    <t>Max Length</t>
   </si>
 </sst>
 </file>
@@ -634,7 +637,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -650,6 +653,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2243,15 +2249,21 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26C3B050-11F0-4CD1-8817-8144CCC481DE}">
-  <dimension ref="A2:C17"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.28515625" customWidth="1"/>
     <col min="2" max="2" width="16.85546875" customWidth="1"/>
     <col min="3" max="3" width="13.5703125" customWidth="1"/>
+    <col min="4" max="4" width="14.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D1" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>29</v>
       </c>
@@ -2262,40 +2274,49 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>23</v>
       </c>
       <c r="B3" t="s">
-        <v>0</v>
+        <v>172</v>
       </c>
       <c r="C3" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D3" s="8">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>24</v>
       </c>
       <c r="B4" t="s">
-        <v>0</v>
+        <v>172</v>
       </c>
       <c r="C4" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D4" s="8">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>25</v>
       </c>
       <c r="B5" t="s">
-        <v>2</v>
+        <v>172</v>
       </c>
       <c r="C5" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D5" s="8">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>26</v>
       </c>
@@ -2306,7 +2327,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>27</v>
       </c>
@@ -2317,7 +2338,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>30</v>
       </c>
@@ -2328,7 +2349,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>89</v>
       </c>
@@ -2339,7 +2360,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>31</v>
       </c>
@@ -2350,7 +2371,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>90</v>
       </c>
@@ -2361,7 +2382,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>16</v>
       </c>
@@ -2372,7 +2393,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>55</v>
       </c>
@@ -2383,7 +2404,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>12</v>
       </c>
@@ -2394,7 +2415,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>13</v>
       </c>
@@ -2405,7 +2426,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>14</v>
       </c>

</xml_diff>

<commit_message>
Fix models and add get expense type name method
</commit_message>
<xml_diff>
--- a/src/main/resources/data/DB.xlsx
+++ b/src/main/resources/data/DB.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28925"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4a765bfb693053ce/Desktop/SecurePrints/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="934" documentId="13_ncr:1_{1D354D38-737B-4D3A-A9B1-62F2684C3BE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3C84ED83-8D10-4D44-97D9-36F6C081E4A0}"/>
+  <xr:revisionPtr revIDLastSave="939" documentId="13_ncr:1_{1D354D38-737B-4D3A-A9B1-62F2684C3BE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5FF397D7-203D-4D41-B158-C5DCFF56FABC}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="810" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="290" uniqueCount="174">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="293" uniqueCount="174">
   <si>
     <t>varchar(30)</t>
   </si>
@@ -170,9 +170,6 @@
   </si>
   <si>
     <t>varchar(60)</t>
-  </si>
-  <si>
-    <t>varchar(15)</t>
   </si>
   <si>
     <t>date</t>
@@ -571,6 +568,9 @@
   </si>
   <si>
     <t>Max Length</t>
+  </si>
+  <si>
+    <t>usr_ip</t>
   </si>
 </sst>
 </file>
@@ -1031,7 +1031,7 @@
         <v>20</v>
       </c>
       <c r="B4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C4" s="1">
         <v>68</v>
@@ -1079,7 +1079,7 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B4" t="s">
         <v>22</v>
@@ -1090,7 +1090,7 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B5" t="s">
         <v>8</v>
@@ -1101,21 +1101,21 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B6" t="s">
         <v>8</v>
       </c>
       <c r="C6" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C7" t="s">
         <v>5</v>
@@ -1123,32 +1123,32 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B8" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C8" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B9" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C9" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B10" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C10" t="s">
         <v>5</v>
@@ -1174,7 +1174,7 @@
         <v>37</v>
       </c>
       <c r="B2" t="s">
-        <v>41</v>
+        <v>0</v>
       </c>
       <c r="C2" t="s">
         <v>4</v>
@@ -1182,7 +1182,7 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B3" t="s">
         <v>2</v>
@@ -1196,7 +1196,7 @@
         <v>39</v>
       </c>
       <c r="B4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C4" t="s">
         <v>5</v>
@@ -1207,7 +1207,7 @@
         <v>38</v>
       </c>
       <c r="B5" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C5" t="s">
         <v>5</v>
@@ -1215,7 +1215,7 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B6" t="s">
         <v>22</v>
@@ -1226,7 +1226,7 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B7" t="s">
         <v>8</v>
@@ -1237,57 +1237,57 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B8" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C8" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B9" t="s">
         <v>8</v>
       </c>
       <c r="C9" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B10" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C10" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B11" t="s">
         <v>40</v>
       </c>
       <c r="C11" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B12" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C12" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
   </sheetData>
@@ -1308,7 +1308,7 @@
   <sheetData>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B2" t="s">
         <v>10</v>
@@ -1319,7 +1319,7 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B3" t="s">
         <v>2</v>
@@ -1330,24 +1330,24 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B4" t="s">
-        <v>41</v>
+        <v>0</v>
       </c>
       <c r="C4" t="s">
         <v>5</v>
       </c>
       <c r="D4" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B5" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C5" t="s">
         <v>5</v>
@@ -1355,7 +1355,7 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B6" t="s">
         <v>8</v>
@@ -1366,7 +1366,7 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B7" t="s">
         <v>8</v>
@@ -1377,18 +1377,18 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B8" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C8" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B9" t="s">
         <v>22</v>
@@ -1399,7 +1399,7 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B10" t="s">
         <v>8</v>
@@ -1410,54 +1410,54 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B11" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C11" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B12" t="s">
         <v>8</v>
       </c>
       <c r="C12" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="B13" t="s">
         <v>40</v>
       </c>
       <c r="C13" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B14" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C14" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B15" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C15" t="s">
         <v>5</v>
@@ -1528,7 +1528,7 @@
         <v>201</v>
       </c>
       <c r="B2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -1536,7 +1536,7 @@
         <v>202</v>
       </c>
       <c r="B3" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -1552,7 +1552,7 @@
         <v>204</v>
       </c>
       <c r="B5" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
   </sheetData>
@@ -1574,7 +1574,7 @@
         <v>301</v>
       </c>
       <c r="B2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -1582,7 +1582,7 @@
         <v>302</v>
       </c>
       <c r="B3" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -1590,7 +1590,7 @@
         <v>303</v>
       </c>
       <c r="B4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -1598,7 +1598,7 @@
         <v>304</v>
       </c>
       <c r="B5" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -1606,7 +1606,7 @@
         <v>305</v>
       </c>
       <c r="B6" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
   </sheetData>
@@ -1627,7 +1627,7 @@
   <sheetData>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B2" s="4" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -1635,10 +1635,10 @@
         <v>401</v>
       </c>
       <c r="B3" t="s">
+        <v>93</v>
+      </c>
+      <c r="C3" t="s">
         <v>94</v>
-      </c>
-      <c r="C3" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -1646,10 +1646,10 @@
         <v>402</v>
       </c>
       <c r="B4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
@@ -1657,10 +1657,10 @@
         <v>403</v>
       </c>
       <c r="B5" t="s">
+        <v>96</v>
+      </c>
+      <c r="C5" t="s">
         <v>97</v>
-      </c>
-      <c r="C5" t="s">
-        <v>98</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -1668,10 +1668,10 @@
         <v>404</v>
       </c>
       <c r="B6" t="s">
+        <v>98</v>
+      </c>
+      <c r="C6" t="s">
         <v>99</v>
-      </c>
-      <c r="C6" t="s">
-        <v>100</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
@@ -1679,10 +1679,10 @@
         <v>405</v>
       </c>
       <c r="B7" t="s">
+        <v>100</v>
+      </c>
+      <c r="C7" t="s">
         <v>101</v>
-      </c>
-      <c r="C7" t="s">
-        <v>102</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
@@ -1690,10 +1690,10 @@
         <v>406</v>
       </c>
       <c r="B8" t="s">
+        <v>102</v>
+      </c>
+      <c r="C8" t="s">
         <v>103</v>
-      </c>
-      <c r="C8" t="s">
-        <v>104</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
@@ -1701,10 +1701,10 @@
         <v>407</v>
       </c>
       <c r="B9" t="s">
+        <v>104</v>
+      </c>
+      <c r="C9" t="s">
         <v>105</v>
-      </c>
-      <c r="C9" t="s">
-        <v>106</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
@@ -1712,10 +1712,10 @@
         <v>408</v>
       </c>
       <c r="B10" t="s">
+        <v>106</v>
+      </c>
+      <c r="C10" t="s">
         <v>107</v>
-      </c>
-      <c r="C10" t="s">
-        <v>108</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
@@ -1723,15 +1723,15 @@
         <v>409</v>
       </c>
       <c r="B11" t="s">
+        <v>108</v>
+      </c>
+      <c r="C11" t="s">
         <v>109</v>
-      </c>
-      <c r="C11" t="s">
-        <v>110</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B13" s="4" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
@@ -1739,10 +1739,10 @@
         <v>501</v>
       </c>
       <c r="B14" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C14" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
@@ -1750,10 +1750,10 @@
         <v>502</v>
       </c>
       <c r="B15" t="s">
+        <v>148</v>
+      </c>
+      <c r="C15" t="s">
         <v>149</v>
-      </c>
-      <c r="C15" t="s">
-        <v>150</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
@@ -1761,13 +1761,13 @@
         <v>503</v>
       </c>
       <c r="B16" t="s">
+        <v>150</v>
+      </c>
+      <c r="C16" t="s">
         <v>151</v>
       </c>
-      <c r="C16" t="s">
+      <c r="D16" t="s">
         <v>152</v>
-      </c>
-      <c r="D16" t="s">
-        <v>153</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
@@ -1775,10 +1775,10 @@
         <v>504</v>
       </c>
       <c r="B17" t="s">
+        <v>153</v>
+      </c>
+      <c r="C17" t="s">
         <v>154</v>
-      </c>
-      <c r="C17" t="s">
-        <v>155</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
@@ -1786,15 +1786,15 @@
         <v>505</v>
       </c>
       <c r="B18" t="s">
+        <v>155</v>
+      </c>
+      <c r="C18" t="s">
         <v>156</v>
-      </c>
-      <c r="C18" t="s">
-        <v>157</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B20" s="4" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
@@ -1802,10 +1802,10 @@
         <v>601</v>
       </c>
       <c r="B21" t="s">
+        <v>111</v>
+      </c>
+      <c r="C21" t="s">
         <v>112</v>
-      </c>
-      <c r="C21" t="s">
-        <v>113</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
@@ -1813,10 +1813,10 @@
         <v>602</v>
       </c>
       <c r="B22" t="s">
+        <v>113</v>
+      </c>
+      <c r="C22" t="s">
         <v>114</v>
-      </c>
-      <c r="C22" t="s">
-        <v>115</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
@@ -1824,10 +1824,10 @@
         <v>603</v>
       </c>
       <c r="B23" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C23" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
@@ -1835,10 +1835,10 @@
         <v>604</v>
       </c>
       <c r="B24" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C24" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
@@ -1846,10 +1846,10 @@
         <v>605</v>
       </c>
       <c r="B25" t="s">
+        <v>117</v>
+      </c>
+      <c r="C25" t="s">
         <v>118</v>
-      </c>
-      <c r="C25" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
@@ -1857,10 +1857,10 @@
         <v>606</v>
       </c>
       <c r="B26" t="s">
+        <v>119</v>
+      </c>
+      <c r="C26" t="s">
         <v>120</v>
-      </c>
-      <c r="C26" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
@@ -1868,10 +1868,10 @@
         <v>607</v>
       </c>
       <c r="B27" t="s">
+        <v>121</v>
+      </c>
+      <c r="C27" t="s">
         <v>122</v>
-      </c>
-      <c r="C27" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
@@ -1879,15 +1879,15 @@
         <v>608</v>
       </c>
       <c r="B28" t="s">
+        <v>123</v>
+      </c>
+      <c r="C28" t="s">
         <v>124</v>
-      </c>
-      <c r="C28" t="s">
-        <v>125</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B30" s="4" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
@@ -1895,7 +1895,7 @@
         <v>701</v>
       </c>
       <c r="B31" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
@@ -1903,7 +1903,7 @@
         <v>702</v>
       </c>
       <c r="B32" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
@@ -1911,7 +1911,7 @@
         <v>703</v>
       </c>
       <c r="B33" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
@@ -1919,12 +1919,12 @@
         <v>704</v>
       </c>
       <c r="B34" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B36" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
@@ -1932,10 +1932,10 @@
         <v>801</v>
       </c>
       <c r="B37" t="s">
+        <v>131</v>
+      </c>
+      <c r="C37" t="s">
         <v>132</v>
-      </c>
-      <c r="C37" t="s">
-        <v>133</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
@@ -1943,10 +1943,10 @@
         <v>802</v>
       </c>
       <c r="B38" t="s">
+        <v>133</v>
+      </c>
+      <c r="C38" t="s">
         <v>134</v>
-      </c>
-      <c r="C38" t="s">
-        <v>135</v>
       </c>
     </row>
     <row r="39" spans="1:4" ht="30" x14ac:dyDescent="0.25">
@@ -1954,13 +1954,13 @@
         <v>803</v>
       </c>
       <c r="B39" s="6" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C39" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="D39" s="5" t="s">
         <v>144</v>
-      </c>
-      <c r="D39" s="5" t="s">
-        <v>145</v>
       </c>
     </row>
     <row r="40" spans="1:4" ht="30" x14ac:dyDescent="0.25">
@@ -1968,18 +1968,18 @@
         <v>804</v>
       </c>
       <c r="B40" s="6" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C40" s="5" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D40" s="5" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B42" s="4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
@@ -1987,10 +1987,10 @@
         <v>901</v>
       </c>
       <c r="B43" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C43" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
@@ -1998,10 +1998,10 @@
         <v>902</v>
       </c>
       <c r="B44" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C44" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
@@ -2009,10 +2009,10 @@
         <v>903</v>
       </c>
       <c r="B45" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C45" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
   </sheetData>
@@ -2035,7 +2035,7 @@
   <sheetData>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B2" t="s">
         <v>8</v>
@@ -2046,7 +2046,7 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B3" t="s">
         <v>40</v>
@@ -2055,15 +2055,15 @@
         <v>5</v>
       </c>
       <c r="D3" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B4" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C4" t="s">
         <v>5</v>
@@ -2071,10 +2071,10 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B5" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C5" t="s">
         <v>5</v>
@@ -2082,7 +2082,7 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B6" t="s">
         <v>3</v>
@@ -2093,7 +2093,7 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B7" t="s">
         <v>2</v>
@@ -2121,7 +2121,7 @@
   <sheetData>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B2" t="s">
         <v>8</v>
@@ -2132,7 +2132,7 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B3" t="s">
         <v>40</v>
@@ -2143,7 +2143,7 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B4" t="s">
         <v>3</v>
@@ -2152,15 +2152,15 @@
         <v>5</v>
       </c>
       <c r="D4" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B5" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C5" t="s">
         <v>5</v>
@@ -2168,10 +2168,10 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>74</v>
+      </c>
+      <c r="B6" t="s">
         <v>75</v>
-      </c>
-      <c r="B6" t="s">
-        <v>76</v>
       </c>
       <c r="C6" t="s">
         <v>5</v>
@@ -2205,10 +2205,10 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>55</v>
+      </c>
+      <c r="B3" t="s">
         <v>56</v>
-      </c>
-      <c r="B3" t="s">
-        <v>57</v>
       </c>
       <c r="C3" t="s">
         <v>5</v>
@@ -2230,13 +2230,13 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B5" t="s">
         <v>11</v>
       </c>
       <c r="C5" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
@@ -2249,7 +2249,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26C3B050-11F0-4CD1-8817-8144CCC481DE}">
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:D18"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.28515625" customWidth="1"/>
@@ -2260,7 +2260,7 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D1" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
@@ -2279,7 +2279,7 @@
         <v>23</v>
       </c>
       <c r="B3" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C3" t="s">
         <v>5</v>
@@ -2293,7 +2293,7 @@
         <v>24</v>
       </c>
       <c r="B4" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C4" t="s">
         <v>5</v>
@@ -2307,10 +2307,10 @@
         <v>25</v>
       </c>
       <c r="B5" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C5" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D5" s="8">
         <v>60</v>
@@ -2324,7 +2324,7 @@
         <v>0</v>
       </c>
       <c r="C6" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
@@ -2346,18 +2346,18 @@
         <v>3</v>
       </c>
       <c r="C8" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B9" t="s">
         <v>11</v>
       </c>
       <c r="C9" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
@@ -2368,18 +2368,18 @@
         <v>3</v>
       </c>
       <c r="C10" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B11" t="s">
         <v>11</v>
       </c>
       <c r="C11" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
@@ -2395,7 +2395,7 @@
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B13" t="s">
         <v>8</v>
@@ -2423,7 +2423,7 @@
         <v>1</v>
       </c>
       <c r="C15" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
@@ -2434,7 +2434,7 @@
         <v>1</v>
       </c>
       <c r="C16" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
@@ -2445,7 +2445,18 @@
         <v>1</v>
       </c>
       <c r="C17" t="s">
-        <v>44</v>
+        <v>43</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>173</v>
+      </c>
+      <c r="B18" t="s">
+        <v>3</v>
+      </c>
+      <c r="C18" t="s">
+        <v>43</v>
       </c>
     </row>
   </sheetData>

</xml_diff>